<commit_message>
Risorse 01-05 rigenerate: ultra-utili, brand AI Osha, no PMI
- Aspetto coerente col sito (Helvetica, titoli navy/ciano, footer aiosha.it su ogni pagina)
- Rebrand "per PMI" -> "per chi lavora"; accenti italiani corretti; firma Aliosha Battaglini + aiosha.it
- R01: 20 domande bilanciate (4x5), punteggio in % equo, "CONCENTRATI sul capitolo X", esempio + piano 7 giorni
- R02: 50 prompt, guida + 5 regole + legenda + tool consigliato per sezione, prompt copiabili
- R03: policy con placeholder uniformi, tabelle livelli dati e ruoli, regola d'oro
- R04: 12 strumenti, valuta unificata, Selettore Guidato con formula funzionante
- R05: ristrutturato (no domande orfane), prezzi allineati a R04
- index.html: conteggio strumenti 7 -> 12

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risorse/Risorsa_04_Confronto_Tool_AI.xlsx
+++ b/risorse/Risorsa_04_Confronto_Tool_AI.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,32 +27,45 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A5F"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="0000838F"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00777777"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0000A8E8"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="0000838F"/>
-      <sz val="11"/>
+      <color rgb="001E3A5F"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="5">
@@ -64,21 +77,21 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000BCD4"/>
+        <fgColor rgb="001E3A5F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000A1F2E"/>
+        <fgColor rgb="00E8F4FD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF9C4"/>
+        <fgColor rgb="00F5A623"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -86,83 +99,41 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CFD8DC"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CFD8DC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CFD8DC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CFD8DC"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CFD8DC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CFD8DC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CFD8DC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CFD8DC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CFD8DC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CFD8DC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -529,36 +500,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AIOsha · Risorsa 04 — Confronto Tool AI</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
+          <t>AI Osha — Risorsa 04 · Confronto Strumenti AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quale strumento per quale uso in PMI</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
+          <t>Quale strumento per quale uso. Voti 1-5. Prezzi indicativi €/mese (lordo IVA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Tool</t>
@@ -596,7 +567,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Qualità output 1-5</t>
+          <t>Qualità 1-5</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -606,7 +577,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Caso d'uso PMI consigliato</t>
+          <t>Caso d'uso consigliato</t>
         </is>
       </c>
     </row>
@@ -634,18 +605,18 @@
       <c r="E5" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="H5" s="6" t="n">
+      <c r="G5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="5" t="n">
         <v>5</v>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Server US, no formazione su dati Plus</t>
+          <t>Server US, no training su dati Plus</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -655,44 +626,44 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Claude (Sonnet 4.6)</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Scrittura/ragionamento</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Voce naturale + analisi documenti</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>No immagini in output</t>
         </is>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G6" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="H6" s="6" t="n">
+      <c r="G6" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>Conserva 30gg, opt-out training</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>Mail clienti, contratti, analisi documenti</t>
         </is>
@@ -722,13 +693,13 @@
       <c r="E7" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="H7" s="5" t="n">
         <v>4</v>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -738,49 +709,49 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Aziende già su Google Workspace</t>
+          <t>Chi è già su Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Perplexity Pro</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Ricerca con fonti</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Risposte con citazioni verificabili</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Non genera contenuti lunghi</t>
         </is>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F8" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="6" t="n">
+      <c r="G8" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H8" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="H8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>Trasparente, no training su input</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>Ricerche di mercato, fact-checking</t>
         </is>
@@ -799,7 +770,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Risposte SOLO su documenti caricati</t>
+          <t>Risposte SOLO sui documenti caricati</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -810,13 +781,13 @@
       <c r="E9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="G9" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="H9" s="5" t="n">
         <v>4</v>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -831,46 +802,48 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Copilot 365</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Office</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Dentro Word/Excel/Outlook/Teams</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Costo per utente alto</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="F10" s="6" t="n">
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Costo per utente</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>22*</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G10" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="G10" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>Tenant aziendale</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>PMI già su Microsoft 365</t>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>Chi è già su Microsoft 365</t>
         </is>
       </c>
     </row>
@@ -882,12 +855,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Video da testo + real-time X</t>
+          <t>Video da testo + real-time</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Generazione video da prompt, tempo reale social</t>
+          <t>Genera video da prompt, tempo reale</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -898,18 +871,18 @@
       <c r="E11" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G11" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="H11" s="6" t="n">
+      <c r="G11" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" s="5" t="n">
         <v>5</v>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Policy dati in evoluzione, verificare per dati sensibili</t>
+          <t>Policy dati in evoluzione: verificare per dati sensibili</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -919,46 +892,46 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>ElevenLabs</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Voce AI</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Cloning vocale + 30 lingue</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Costo crescente per minuti</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="n">
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Costo per minuti</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="F12" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="G12" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="H12" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>Conservazione audio limitata</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>Audiolibri, podcast aziendali, IVR</t>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>Audiolibri, podcast, IVR</t>
         </is>
       </c>
     </row>
@@ -986,13 +959,13 @@
       <c r="E13" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F13" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="H13" s="6" t="n">
+      <c r="G13" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" s="5" t="n">
         <v>3</v>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1007,44 +980,44 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Midjourney</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Immagini AI</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Estetica forte, look professionale</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Solo Discord o web</t>
         </is>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="F14" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="G14" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="H14" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>Input visibili a community se public</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>Input visibili alla community se public</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>Mood board, immagini social premium</t>
         </is>
@@ -1053,7 +1026,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>DALL-E 3 (in ChatGPT)</t>
+          <t>DALL·E 3 (in ChatGPT)</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1076,13 +1049,13 @@
           <t>incluso</t>
         </is>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F15" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="H15" s="6" t="n">
+      <c r="G15" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" s="5" t="n">
         <v>4</v>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1097,92 +1070,59 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Make.com / n8n</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Automazioni</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Collega AI a Gmail, CRM, Excel</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Curva di apprendimento</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>10-30</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="G16" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="H16" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>10–30</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>n8n self-hosted = 100% controllato</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>Workflow agentici, lead routing</t>
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>* Copilot 365: prezzo per utente. Versioni modelli aggiornate ad aprile 2026.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
-  </mergeCells>
-  <conditionalFormatting sqref="F5:F16">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="num" val="1"/>
-        <cfvo type="num" val="3"/>
-        <cfvo type="num" val="5"/>
-        <color rgb="00FFCDD2"/>
-        <color rgb="00FFF59D"/>
-        <color rgb="00C8E6C9"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G5:G16">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="num" val="1"/>
-        <cfvo type="num" val="3"/>
-        <cfvo type="num" val="5"/>
-        <color rgb="00FFCDD2"/>
-        <color rgb="00FFF59D"/>
-        <color rgb="00C8E6C9"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H16">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="num" val="1"/>
-        <cfvo type="num" val="3"/>
-        <cfvo type="num" val="5"/>
-        <color rgb="00FFCDD2"/>
-        <color rgb="00FFF59D"/>
-        <color rgb="00C8E6C9"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1193,132 +1133,153 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AIOsha · Selettore guidato</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
+          <t>AI Osha — Selettore guidato</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rispondi con SI/NO e leggi la raccomandazione finale</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+          <t>Scegli SI/NO nella colonna B. La raccomandazione si aggiorna da sola in fondo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Domanda</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Risposta (SI/NO)</t>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Risposta</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Usi già Microsoft 365 in azienda?</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>1. Usi già Microsoft 365 (Word/Excel/Outlook/Teams)?</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Usi già Google Workspace?</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>2. Usi già Google Workspace (Gmail/Docs/Drive)?</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Produci video brevi per social con frequenza?</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>3. Il tuo lavoro è soprattutto scrivere (testi lunghi)?</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Ti serve voce AI / podcast?</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>4. Produci video brevi per i social con frequenza?</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Vuoi automazioni che colleghino più tool?</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>5. Ti serve ricerca con fonti verificabili?</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Ti serve ricerca con fonti verificabili?</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>6. Ti serve voce AI / podcast?</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Raccomandazione AIOsha</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="n"/>
-    </row>
-    <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="9">
-        <f>IF(B5="SI","Copilot 365 + Claude per scrittura. ",IF(B6="SI","Gemini + NotebookLM. ",IF(B7="SI","Grok SuperGrok per generazione video. ","ChatGPT Plus + Claude come combinazione di base. ")))</f>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>7. Vuoi automazioni che colleghino più tool?</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>LA TUA RACCOMANDAZIONE</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr"/>
+    </row>
+    <row r="14" ht="46" customHeight="1">
+      <c r="A14" s="14">
+        <f>"Principale: "&amp;IF(B5="SI","Microsoft Copilot 365 (22 €/mese)",IF(B6="SI","Gemini Advanced (22 €/mese)",IF(B7="SI","Claude Pro (20 €/mese)","ChatGPT Plus (20 €/mese)")))&amp;IF(B8="SI","  +  Grok video (30 €)","")&amp;IF(B9="SI","  +  Perplexity Pro (20 €)","")&amp;IF(B10="SI","  +  ElevenLabs (22 €)","")&amp;IF(B11="SI","  +  Make/n8n (10–30 €)","")</f>
         <v/>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Consiglio: parti da 1 strumento principale. Aggiungi 1 specialista solo dopo 60 giorni.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A12:B12"/>
+  <mergeCells count="1">
+    <mergeCell ref="A14:B14"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B5 B6 B7 B8 B9 B10 B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"SI,NO"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>